<commit_message>
Leads: 2026-10-19 15:35 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-19.xlsx
+++ b/output/leads_2026-10-19.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Elite Mechanical</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>elitemechanical.org</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://elitemechanical.org/about-us/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Elite Mechanical</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>mike.burriss@elitemechanical.org</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(775) 447-2224</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Sparks NV</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>82</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>HVAC contractor Sparks NV</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-19 15:39 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-19.xlsx
+++ b/output/leads_2026-10-19.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,126 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Atlanta Roofing Installers</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>atlantaroofinginstallers.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://atlantaroofinginstallers.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>How Atlanta</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>sbesupply@gmail.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(678) 693-9767</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Atlanta GA</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roofing contractor Atlanta GA</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Fort Wayne Roofing — A Tecta America Co.</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>fortwayneroofing.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.fortwayneroofing.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Residential Residential</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>service.fortwayne@tectaamerica.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(260) 422-9529</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>residential roofing company Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-19 15:41 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-19.xlsx
+++ b/output/leads_2026-10-19.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -803,6 +803,62 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>O'Brien's HVAC Company</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>obrienshvac.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://obrienshvac.com/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>obrienshvacstacey@gmail.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>843-460-0269</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Charleston SC</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>86</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>heating and cooling company Charleston SC</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-19 20:58 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-19.xlsx
+++ b/output/leads_2026-10-19.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -824,7 +824,6 @@
           <t>https://obrienshvac.com/</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>obrienshvacstacey@gmail.com</t>
@@ -854,6 +853,66 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Des Moines Drain &amp; Sewer</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>desmoinesdrainandsewer.org</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://desmoinesdrainandsewer.org/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Owner Paul</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>unclogger50313@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(515) 289-2837</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Des Moines IA</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>drain cleaning service Des Moines IA</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-19 21:02 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-19.xlsx
+++ b/output/leads_2026-10-19.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -918,6 +918,66 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Aurora Plumbing Pros</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>auroraplumbers.net</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://auroraplumbers.net/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Right The</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>info@auroraplumbers.net</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(303) 963-4900</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>emergency plumber Aurora CO</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-19 21:06 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-19.xlsx
+++ b/output/leads_2026-10-19.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -978,6 +978,66 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Three Stone</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>threestone.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://threestone.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Home Residential</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@threestone.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(615) 434-3333</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Franklin TN</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roof repair company Franklin TN</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-19 21:08 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-19.xlsx
+++ b/output/leads_2026-10-19.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1038,6 +1038,66 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Furnace Repair &amp; HVAC Contractor Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>mountainclimatehvac.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://mountainclimatehvac.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Real Reviews</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>7196634483@tmomail.net</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(719) 663-4483</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>HVAC contractor Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-19 21:14 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-19.xlsx
+++ b/output/leads_2026-10-19.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1098,6 +1098,58 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Greater Burlington Plumbing &amp; HVAC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>burlingtonvtplumbinghvac.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://burlingtonvtplumbinghvac.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>corrections@burlingtonvtplumbinghvac.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Burlington VT</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>66</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>plumbing company Burlington VT</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-19 21:15 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-19.xlsx
+++ b/output/leads_2026-10-19.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1119,13 +1119,11 @@
           <t>https://burlingtonvtplumbinghvac.com/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>corrections@burlingtonvtplumbinghvac.com</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Burlington VT</t>
@@ -1145,6 +1143,66 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Drain Works Inc.</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>michigandrainworks.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://michigandrainworks.com/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Taylor Burrows</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>service@michigandrainworks.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>517.896.7910</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Lansing MI</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>drain cleaning service Lansing MI</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-19 21:18 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-19.xlsx
+++ b/output/leads_2026-10-19.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1208,6 +1208,62 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Roofing Services | Hale Roofing | Bowling Green, KY</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>haleroofingky.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.haleroofingky.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>haleroofing@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(270) 842-2989</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Bowling Green KY</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>roof replacement Bowling Green KY</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>